<commit_message>
Rework payroll deductions; add run rollback and bank export summary
Advances now mirror loans: each carries an outstanding_amount balance
(new advance_repayments ledger), drawn down on approve and carried over
to later payrolls instead of being auto-deducted in full.

- Payroll draft pre-fills both loan and advance deductions with each
  employee's outstanding balance; edit down before approving
- Delete an approved run: reverses its loan repayments and advance
  draw-downs (balances restored, ledgers cleared), freeing the month
  to be generated again
- Excel export adds a Salary Disbursement Summary table (Phone Number,
  Amount, Comment) as the bank's upload payload — Amount is a plain
  stored value equal to Net Salary, Comment is 'salary'
- Schema: add salary_advances.outstanding_amount and advance_repayments
  table (Alembic revisions a1b2c3d4e5f6, b2c3d4e5f6a7
</commit_message>
<xml_diff>
--- a/excel/payroll_export.xlsx
+++ b/excel/payroll_export.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leonj\OneDrive\Desktop\payroll-system\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\leonj\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D78B743A-F564-4F57-BC6C-56F5BB5D6C43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91CA8F94-0673-4E2C-90C0-B49C73ACFEDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,12 +56,24 @@
         </r>
       </text>
     </comment>
+    <comment ref="B37" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0000-000002000000}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t>Format only — Phone and Amount are formulas referencing the detail table above (e.g. B39=B6), so this section stays in sync automatically as rows are filled in. Amount is the employee's Net Salary; Comment is always the literal text 'salary'. Confirm this three-column shape against the actual bank/M-Pesa bulk-upload requirement before treating it as final.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="15">
   <si>
     <t>Monthly Payroll Export</t>
   </si>
@@ -94,6 +106,18 @@
   </si>
   <si>
     <t>Check: Gross - Deductions = Net</t>
+  </si>
+  <si>
+    <t>Bank / M-Pesa Bulk Payment Summary — pulled from the table above</t>
+  </si>
+  <si>
+    <t>Amount (KES)</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>salary</t>
   </si>
 </sst>
 </file>
@@ -210,8 +234,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -223,9 +250,8 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -490,7 +516,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F63"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -501,373 +527,727 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
+      <c r="F3" s="1"/>
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="2"/>
-      <c r="B6" s="3"/>
-      <c r="C6" s="4"/>
-      <c r="D6" s="4"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="5">
+      <c r="A6" s="5"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="7"/>
+      <c r="E6" s="7"/>
+      <c r="F6" s="8">
         <f t="shared" ref="F6:F30" si="0">C6-D6-E6</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="2"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="5">
+      <c r="A7" s="5"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="7"/>
+      <c r="E7" s="7"/>
+      <c r="F7" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="2"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="4"/>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
-      <c r="F8" s="5">
+      <c r="A8" s="5"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="7"/>
+      <c r="D8" s="7"/>
+      <c r="E8" s="7"/>
+      <c r="F8" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="2"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="5">
+      <c r="A9" s="5"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="2"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="5">
+      <c r="A10" s="5"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="2"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="5">
+      <c r="A11" s="5"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="2"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="5">
+      <c r="A12" s="5"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="2"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="5">
+      <c r="A13" s="5"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="2"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="5">
+      <c r="A14" s="5"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="2"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="5">
+      <c r="A15" s="5"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="2"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="5">
+      <c r="A16" s="5"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="2"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="5">
+      <c r="A17" s="5"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" s="2"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="5">
+      <c r="A18" s="5"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="2"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="5">
+      <c r="A19" s="5"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="2"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="5">
+      <c r="A20" s="5"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="2"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="5">
+      <c r="A21" s="5"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="2"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="5">
+      <c r="A22" s="5"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="2"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="5">
+      <c r="A23" s="5"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="2"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="5">
+      <c r="A24" s="5"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="2"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="5">
+      <c r="A25" s="5"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="2"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="5">
+      <c r="A26" s="5"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="2"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="5">
+      <c r="A27" s="5"/>
+      <c r="B27" s="6"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="2"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="5">
+      <c r="A28" s="5"/>
+      <c r="B28" s="6"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="2"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="4"/>
-      <c r="D29" s="4"/>
-      <c r="E29" s="4"/>
-      <c r="F29" s="5">
+      <c r="A29" s="5"/>
+      <c r="B29" s="6"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="2"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="4"/>
-      <c r="D30" s="4"/>
-      <c r="E30" s="4"/>
-      <c r="F30" s="5">
+      <c r="A30" s="5"/>
+      <c r="B30" s="6"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="8">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="6" t="s">
+      <c r="A31" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="7">
+      <c r="B31" s="9"/>
+      <c r="C31" s="10">
         <f>SUM(C6:C30)</f>
         <v>0</v>
       </c>
-      <c r="D31" s="7">
+      <c r="D31" s="10">
         <f>SUM(D6:D30)</f>
         <v>0</v>
       </c>
-      <c r="E31" s="7">
+      <c r="E31" s="10">
         <f>SUM(E6:E30)</f>
         <v>0</v>
       </c>
-      <c r="F31" s="7">
+      <c r="F31" s="10">
         <f>SUM(F6:F30)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="8" t="s">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A33" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C33" s="9">
+      <c r="C33" s="12">
         <f>(D31+E31)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="8" t="s">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A34" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="C34" s="8" t="str">
+      <c r="C34" s="11" t="str">
         <f>IF(ROUND(C31-D31-E31-F31,2)=0,"OK","MISMATCH")</f>
         <v>OK</v>
       </c>
     </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B36" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+    </row>
+    <row r="37" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B37" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B38" s="13">
+        <f t="shared" ref="B38:B62" si="1">B6</f>
+        <v>0</v>
+      </c>
+      <c r="C38" s="8">
+        <f t="shared" ref="C38:C62" si="2">F6</f>
+        <v>0</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B39" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C39" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B40" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C40" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B41" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C41" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B42" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C42" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B43" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C43" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B44" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C44" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B45" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C45" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D45" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B46" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C46" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D46" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B47" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C47" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D47" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B48" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C48" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D48" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="49" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B49" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C49" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D49" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="50" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B50" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C50" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D50" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="51" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B51" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C51" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="52" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B52" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C52" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D52" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="53" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B53" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C53" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D53" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="54" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B54" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C54" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D54" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="55" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B55" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C55" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D55" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="56" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B56" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C56" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D56" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="57" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B57" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C57" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D57" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="58" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B58" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C58" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D58" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="59" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B59" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C59" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D59" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="60" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B60" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C60" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D60" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="61" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B61" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C61" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D61" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="62" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B62" s="13">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C62" s="8">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="D62" s="5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="63" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B63" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C63" s="10">
+        <f>SUM(C38:C62)</f>
+        <v>0</v>
+      </c>
+      <c r="D63" s="14"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A3:F3"/>
+    <mergeCell ref="B36:D36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>